<commit_message>
Add decision dropdown columns to comparison table
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017M1hoKEKMcmLsUKHM8fd7N
</commit_message>
<xml_diff>
--- a/output/comparison_table.xlsx
+++ b/output/comparison_table.xlsx
@@ -39,7 +39,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +49,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF263B53"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -73,6 +78,9 @@
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -440,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -449,6 +457,8 @@
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,6 +492,16 @@
           <t>הערות לאישור המחבר</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ההחלטה</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>הערה (אם בחרת "אחר")</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -554,6 +574,8 @@
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -800,6 +822,8 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -918,6 +942,8 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1045,6 +1071,8 @@
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1117,6 +1145,8 @@
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1285,6 +1315,8 @@
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1357,6 +1389,8 @@
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1955,6 +1989,8 @@
           <t>פסקה משובשת (כולל המילה "כאילדדדו") שוחזרה לפי ההקשר; נא לאשר את הנוסח ואת הרמז הדרשני.</t>
         </is>
       </c>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2027,6 +2063,8 @@
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2283,6 +2321,8 @@
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2625,6 +2665,8 @@
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3714,6 +3756,8 @@
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3891,6 +3935,8 @@
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4215,6 +4261,8 @@
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4278,6 +4326,8 @@
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4437,6 +4487,8 @@
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4628,6 +4680,8 @@
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4787,6 +4841,8 @@
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4964,6 +5020,8 @@
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5137,6 +5195,8 @@
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5186,6 +5246,8 @@
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5267,6 +5329,8 @@
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6206,6 +6270,8 @@
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6406,6 +6472,8 @@
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6763,6 +6831,8 @@
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7105,6 +7175,8 @@
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7241,6 +7313,8 @@
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7446,6 +7520,8 @@
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7518,6 +7594,8 @@
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7691,6 +7769,8 @@
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -7923,6 +8003,8 @@
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -7995,6 +8077,8 @@
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8296,6 +8380,8 @@
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8606,6 +8692,8 @@
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -8701,6 +8789,8 @@
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -8841,6 +8931,8 @@
           <t>הנוסח "וכתב שלא יהיה אלא ספק" נראה משובש; תוקן למשמעות המשוערת ("אפילו אם אינו אלא ספק"). נא לאשר מול דברי האשל אברהם.</t>
         </is>
       </c>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9005,6 +9097,8 @@
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9356,6 +9450,8 @@
           <t>"וזה כמו האסלא של ימינו" – ייתכן שחסרה המילה "אינו" ("וזה אינו כמו האסלה של ימינו"), שכן ההקשר הוא הבדל בין בית הכסא של פעם לשל ימינו. הנוסח לא שונה מהותית; נא לאשר.</t>
         </is>
       </c>
+      <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9419,6 +9515,8 @@
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -9486,6 +9584,8 @@
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -9947,6 +10047,8 @@
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10023,6 +10125,8 @@
           <t>השאלה כוללת קטע לא ברור: "או בעד בדיקה" (אולי "בעת בדיקתן"?). תוקן רק "שיש בה" → "שיש בהן"; נא לברר את כוונת המחבר.</t>
         </is>
       </c>
+      <c r="G43" s="4" t="n"/>
+      <c r="H43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10228,6 +10332,8 @@
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -10405,6 +10511,8 @@
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -10477,6 +10585,8 @@
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -10645,6 +10755,8 @@
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="4" t="n"/>
+      <c r="H47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -10717,6 +10829,8 @@
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -10926,6 +11040,8 @@
           <t>הפסקה נקטעת באמצע משפט ("ס"ק סא") וממשיכה בפסקה נפרדת, ויש בהמשך נוסח משובש ("כתב בשם הזוהר כתב דלא יברך... מקום כתב להקל כשאים לו מים"). לא איחדתי את הפסקאות (כדי לשמור על המבנה), אך נא לאשר את איחודן ואת הנוסח המשוחזר, וכן את מראה המקום "ס"ק סא".</t>
         </is>
       </c>
+      <c r="G49" s="4" t="n"/>
+      <c r="H49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -10998,6 +11114,8 @@
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -11111,6 +11229,8 @@
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -11183,6 +11303,8 @@
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="4" t="n"/>
+      <c r="H52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -11428,6 +11550,8 @@
           <t>שם הספר "ספר החסדים" טעון בדיקה (ייתכן "ספר חסידים"); שונה רק "מספר" ל"בספר" ולא נגעתי בשם הספר ובמראה המקום.</t>
         </is>
       </c>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -11633,6 +11757,8 @@
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -11769,6 +11895,8 @@
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="4" t="n"/>
+      <c r="H55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -12189,6 +12317,8 @@
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -12325,6 +12455,8 @@
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -12603,6 +12735,8 @@
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -12666,6 +12800,8 @@
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -12839,6 +12975,8 @@
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -12934,6 +13072,8 @@
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="4" t="n"/>
+      <c r="H61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -13240,8 +13380,15 @@
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="G2:G62" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="בחירה" error="נא לבחור מהרשימה" promptTitle="ההחלטה" prompt="בחר: להשאיר את המקור / להשאיר את השינויים / אחר" type="list">
+      <formula1>"להשאיר את המקור,להשאיר את השינויים,אחר"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13252,7 +13399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13261,6 +13408,8 @@
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13294,6 +13443,16 @@
           <t>הערות לאישור המחבר</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ההחלטה</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>הערה (אם בחרת "אחר")</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -13375,6 +13534,8 @@
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -13470,6 +13631,8 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -13652,6 +13815,8 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -13733,6 +13898,8 @@
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -13837,6 +14004,8 @@
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -13909,6 +14078,8 @@
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -14113,6 +14284,8 @@
           <t>"המ"א" שונה ל"המג"א" לפי ההמשך באותה הערה (מג"א סימן צא סק"ג); נא לוודא.</t>
         </is>
       </c>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -14194,6 +14367,8 @@
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -14257,6 +14432,8 @@
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -14375,6 +14552,8 @@
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -14543,6 +14722,8 @@
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -14592,6 +14773,8 @@
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -14696,6 +14879,8 @@
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -14768,6 +14953,8 @@
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -14840,6 +15027,8 @@
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -14912,6 +15101,8 @@
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -14975,6 +15166,8 @@
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -15285,6 +15478,8 @@
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -15357,6 +15552,8 @@
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -15539,6 +15736,8 @@
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -15643,6 +15842,8 @@
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -15715,6 +15916,8 @@
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -15842,6 +16045,8 @@
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -15905,6 +16110,8 @@
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -15986,6 +16193,8 @@
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -16058,6 +16267,8 @@
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -16130,6 +16341,8 @@
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -16193,6 +16406,8 @@
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -16288,8 +16503,15 @@
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="G2:G30" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="בחירה" error="נא לבחור מהרשימה" promptTitle="ההחלטה" prompt="בחר: להשאיר את המקור / להשאיר את השינויים / אחר" type="list">
+      <formula1>"להשאיר את המקור,להשאיר את השינויים,אחר"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16300,7 +16522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16308,6 +16530,8 @@
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16336,6 +16560,16 @@
           <t>הערה לאישור המחבר</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ההחלטה</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>הערה (אם בחרת "אחר")</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -16929,6 +17163,8 @@
           <t>פסקה משובשת (כולל המילה "כאילדדדו") שוחזרה לפי ההקשר; נא לאשר את הנוסח ואת הרמז הדרשני.</t>
         </is>
       </c>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -17032,6 +17268,8 @@
           <t>הנוסח "וכתב שלא יהיה אלא ספק" נראה משובש; תוקן למשמעות המשוערת ("אפילו אם אינו אלא ספק"). נא לאשר מול דברי האשל אברהם.</t>
         </is>
       </c>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -17103,6 +17341,8 @@
           <t>"וזה כמו האסלא של ימינו" – ייתכן שחסרה המילה "אינו" ("וזה אינו כמו האסלה של ימינו"), שכן ההקשר הוא הבדל בין בית הכסא של פעם לשל ימינו. הנוסח לא שונה מהותית; נא לאשר.</t>
         </is>
       </c>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -17174,6 +17414,8 @@
           <t>השאלה כוללת קטע לא ברור: "או בעד בדיקה" (אולי "בעת בדיקתן"?). תוקן רק "שיש בה" → "שיש בהן"; נא לברר את כוונת המחבר.</t>
         </is>
       </c>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -17378,6 +17620,8 @@
           <t>הפסקה נקטעת באמצע משפט ("ס"ק סא") וממשיכה בפסקה נפרדת, ויש בהמשך נוסח משובש ("כתב בשם הזוהר כתב דלא יברך... מקום כתב להקל כשאים לו מים"). לא איחדתי את הפסקאות (כדי לשמור על המבנה), אך נא לאשר את איחודן ואת הנוסח המשוחזר, וכן את מראה המקום "ס"ק סא".</t>
         </is>
       </c>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -17449,6 +17693,8 @@
           <t>שם הספר "ספר החסדים" טעון בדיקה (ייתכן "ספר חסידים"); שונה רק "מספר" ל"בספר" ולא נגעתי בשם הספר ובמראה המקום.</t>
         </is>
       </c>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -17520,8 +17766,15 @@
           <t>"המ"א" שונה ל"המג"א" לפי ההמשך באותה הערה (מג"א סימן צא סק"ג); נא לוודא.</t>
         </is>
       </c>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="בחירה" error="נא לבחור מהרשימה" promptTitle="ההחלטה" prompt="בחר: להשאיר את המקור / להשאיר את השינויים / אחר" type="list">
+      <formula1>"להשאיר את המקור,להשאיר את השינויים,אחר"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17532,12 +17785,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17556,6 +17811,16 @@
           <t>מה לאשר</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ההחלטה</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>הערה (אם בחרת "אחר")</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -17573,6 +17838,8 @@
           <t>בהמשך המשפט נאמר שבכל אופן חולץ השמאל תחילה, בעוד שתחילת המשפט עוסקת בחליצת ימין תחילה – נראה שנפל ט"ס (אולי "ילבש הימין תחילה"). לא שונה.</t>
         </is>
       </c>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -17590,6 +17857,8 @@
           <t>הניסוח והקישור למימרא "מי שאכל שום וריחו נודף יחזור ויאכל" אינם ברורים (נראה שחסרה מילת הסבר). לא שונה – נא לנסח.</t>
         </is>
       </c>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -17607,6 +17876,8 @@
           <t>יש לאחד את שתי הפסקאות (91 ו-92), ולברר את מראה המקום "ס"ק סא". המבנה לא שונה כדי לשמור על העימוד. הנוסח המשובש בפסקה 92 שוחזר ודווח בגיליון השינויים המהותיים.</t>
         </is>
       </c>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -17624,6 +17895,8 @@
           <t>נשמר כפי שהוא. נא לאשר שזו הכוונה (שאלות ללא תשובה נפרדת).</t>
         </is>
       </c>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -17641,6 +17914,8 @@
           <t>מראה המקום לא שונה (ייתכן: סימן ב, סעיף קטן ג). נא לוודא ולאחד את צורת הכתיבה.</t>
         </is>
       </c>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -17658,6 +17933,8 @@
           <t>"ביה"כ" בהקשר זה כנראה בית הכסא (בדרך כלל "ביהכ"ס"; "ביה"כ" משמעו לרוב בית הכנסת). לא שונה – נא לאשר.</t>
         </is>
       </c>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -17675,6 +17952,8 @@
           <t>נשמר הכתיב השכיח במסמך ("ענין", "בודאי", "דוקא", "מדת", "כיון"), והמופעים החריגים בגוף דברי המחבר הותאמו (למשל מצווה→מצוה). לא אוחד: תפלה/תפילה ותחלה/תחילה, כדי לא לפגוע בציטוטים. נא להכריע בכלל אחד.</t>
         </is>
       </c>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -17692,8 +17971,15 @@
           <t>ציטוטים לא שונו (למעט פיסוק מינימלי בלשון המחבר שמסביב), כנדרש – ללא אימות מול המקור.</t>
         </is>
       </c>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D9" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="בחירה" error="נא לבחור מהרשימה" promptTitle="ההחלטה" prompt="בחר: להשאיר את המקור / להשאיר את השינויים / אחר" type="list">
+      <formula1>"להשאיר את המקור,להשאיר את השינויים,אחר"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>